<commit_message>
feat: REST import/export handlers, Bruno test suite (48 tests), app restructure
- Add REST import/export handlers bypassing gRPC-gateway for file upload/download
- Add HTTP auth/permission middleware for REST endpoints
- Extract setupGRPCGateway() and setupHTTPRoutes() from run.go
- Add 48-test Bruno suite (86 assertions) with cleanup scripts
- Fix import: correct Excel column headers, add 'server_name' alias
- Fix update_ip_conflict: real 2-server scenario → 409
- Add import_truly_empty test for ErrEmptyFile (400)
</commit_message>
<xml_diff>
--- a/bruno/testdata/servers.xlsx
+++ b/bruno/testdata/servers.xlsx
@@ -16,10 +16,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
-    <t>server_name</t>
-  </si>
-  <si>
-    <t>ipv4</t>
+    <t>Server Name</t>
+  </si>
+  <si>
+    <t>IPv4</t>
   </si>
   <si>
     <t>import-srv-01</t>

</xml_diff>